<commit_message>
Template: update date format hints to show DD.MM.YYYY and DD/MM/YYYY accepted
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/fleet-import-template.xlsx
+++ b/public/templates/fleet-import-template.xlsx
@@ -455,22 +455,22 @@
         <v>Odometer (km)</v>
       </c>
       <c r="L1" t="str">
-        <v>Gov Inspection Last (DD/MM/YYYY)</v>
+        <v>Gov Inspection Last (date)</v>
       </c>
       <c r="M1" t="str">
-        <v>Gov Inspection Next (DD/MM/YYYY)</v>
+        <v>Gov Inspection Next (date)</v>
       </c>
       <c r="N1" t="str">
-        <v>Service Last (DD/MM/YYYY)</v>
+        <v>Service Last (date)</v>
       </c>
       <c r="O1" t="str">
-        <v>Service Next (DD/MM/YYYY)</v>
+        <v>Service Next (date)</v>
       </c>
       <c r="P1" t="str">
         <v>Insurance Number</v>
       </c>
       <c r="Q1" t="str">
-        <v>Insurance Valid Until (DD/MM/YYYY)</v>
+        <v>Insurance Valid Until (date)</v>
       </c>
       <c r="R1" t="str">
         <v>Notes</v>
@@ -511,22 +511,22 @@
         <v>85000</v>
       </c>
       <c r="L2" t="str">
-        <v>15/03/2024</v>
+        <v>15.03.2024</v>
       </c>
       <c r="M2" t="str">
-        <v>15/03/2026</v>
+        <v>15.03.2026</v>
       </c>
       <c r="N2" t="str">
-        <v>10/01/2024</v>
+        <v>10.01.2024</v>
       </c>
       <c r="O2" t="str">
-        <v>10/01/2025</v>
+        <v>10.01.2025</v>
       </c>
       <c r="P2" t="str">
         <v>POL-12345678</v>
       </c>
       <c r="Q2" t="str">
-        <v>31/12/2025</v>
+        <v>31.12.2025</v>
       </c>
       <c r="R2" t="str">
         <v>Airport delivery key in glove box</v>
@@ -570,7 +570,7 @@
         <v/>
       </c>
       <c r="M3" t="str">
-        <v>01/06/2026</v>
+        <v>01.06.2026</v>
       </c>
       <c r="N3" t="str">
         <v/>
@@ -744,7 +744,7 @@
         <v>no</v>
       </c>
       <c r="C13" t="str">
-        <v>DD/MM/YYYY</v>
+        <v>Date: DD.MM.YYYY or DD/MM/YYYY or YYYY-MM-DD  (e.g. 20.05.2027 or 20/05/2027)</v>
       </c>
     </row>
     <row r="14">
@@ -755,7 +755,7 @@
         <v>no</v>
       </c>
       <c r="C14" t="str">
-        <v>DD/MM/YYYY</v>
+        <v>Date: DD.MM.YYYY or DD/MM/YYYY or YYYY-MM-DD  (e.g. 20.05.2027 or 20/05/2027)</v>
       </c>
     </row>
     <row r="15">
@@ -766,7 +766,7 @@
         <v>no</v>
       </c>
       <c r="C15" t="str">
-        <v>DD/MM/YYYY</v>
+        <v>Date: DD.MM.YYYY or DD/MM/YYYY or YYYY-MM-DD  (e.g. 20.05.2027 or 20/05/2027)</v>
       </c>
     </row>
     <row r="16">
@@ -777,7 +777,7 @@
         <v>no</v>
       </c>
       <c r="C16" t="str">
-        <v>DD/MM/YYYY</v>
+        <v>Date: DD.MM.YYYY or DD/MM/YYYY or YYYY-MM-DD  (e.g. 20.05.2027 or 20/05/2027)</v>
       </c>
     </row>
     <row r="17">
@@ -799,7 +799,7 @@
         <v>no</v>
       </c>
       <c r="C18" t="str">
-        <v>DD/MM/YYYY</v>
+        <v>Date: DD.MM.YYYY or DD/MM/YYYY or YYYY-MM-DD  (e.g. 20.05.2027 or 20/05/2027)</v>
       </c>
     </row>
     <row r="19">

</xml_diff>